<commit_message>
all datas on it
</commit_message>
<xml_diff>
--- a/annotation/a554.xlsx
+++ b/annotation/a554.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,36 @@
           <t>id</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>kalima_text</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>num_sora</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sora_name_ar</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>aya_no</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>kalima_text_emlaey</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -469,6 +499,30 @@
       <c r="F2" t="n">
         <v>1</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>يَٰٓأَيُّهَا</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>62</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ياأيها</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -489,6 +543,30 @@
       <c r="F3" t="n">
         <v>2</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ٱلَّذِينَ</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>62</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>9</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>الذين</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -509,6 +587,30 @@
       <c r="F4" t="n">
         <v>3</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ءَامَنُوٓاْ</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>62</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>آمنوا</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -529,6 +631,30 @@
       <c r="F5" t="n">
         <v>4</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>إِذَا</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>62</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>9</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>إذا</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -549,6 +675,30 @@
       <c r="F6" t="n">
         <v>5</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>نُودِيَ</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>62</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>نودي</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -569,6 +719,30 @@
       <c r="F7" t="n">
         <v>6</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>لِلصَّلَوٰةِ</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>62</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>9</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>للصلاة</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -589,6 +763,30 @@
       <c r="F8" t="n">
         <v>7</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>مِن</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>62</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>9</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>من</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -609,6 +807,30 @@
       <c r="F9" t="n">
         <v>8</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>يَوۡمِ</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>62</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>9</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>يوم</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -629,6 +851,30 @@
       <c r="F10" t="n">
         <v>9</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ٱلۡجُمُعَةِ</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>62</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>الجمعة</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -649,6 +895,30 @@
       <c r="F11" t="n">
         <v>10</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>فَٱسۡعَوۡاْ</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>62</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>9</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>فاسعوا</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -669,6 +939,30 @@
       <c r="F12" t="n">
         <v>11</v>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>إِلَىٰ</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>62</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>9</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>إلى</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -689,6 +983,30 @@
       <c r="F13" t="n">
         <v>12</v>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ذِكۡرِ</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>62</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>9</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ذكر</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -709,6 +1027,30 @@
       <c r="F14" t="n">
         <v>13</v>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ٱللَّهِ</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>62</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>9</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>الله</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -729,6 +1071,30 @@
       <c r="F15" t="n">
         <v>14</v>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>وَذَرُواْ</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>62</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>9</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>وذروا</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -749,6 +1115,30 @@
       <c r="F16" t="n">
         <v>15</v>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ٱلۡبَيۡعَۚ</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>62</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>9</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>البيع</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -769,6 +1159,30 @@
       <c r="F17" t="n">
         <v>16</v>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ذَٰلِكُمۡ</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>62</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>9</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ذلكم</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -789,6 +1203,30 @@
       <c r="F18" t="n">
         <v>17</v>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>خَيۡرٞ</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>62</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>9</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>خير</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -809,6 +1247,30 @@
       <c r="F19" t="n">
         <v>18</v>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>لَّكُمۡ</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>62</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>9</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>لكم</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -829,6 +1291,30 @@
       <c r="F20" t="n">
         <v>19</v>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>إِن</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>62</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>9</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>إن</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -849,6 +1335,30 @@
       <c r="F21" t="n">
         <v>20</v>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>كُنتُمۡ</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>62</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>9</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>كنتم</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -869,6 +1379,30 @@
       <c r="F22" t="n">
         <v>21</v>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>تَعۡلَمُونَ</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>62</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>9</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>تعلمون</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -889,6 +1423,30 @@
       <c r="F23" t="n">
         <v>23</v>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>فَإِذَا</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>62</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>10</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>فإذا</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -909,6 +1467,30 @@
       <c r="F24" t="n">
         <v>24</v>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>قُضِيَتِ</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>62</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>10</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>قضيت</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -929,6 +1511,30 @@
       <c r="F25" t="n">
         <v>25</v>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>ٱلصَّلَوٰةُ</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>62</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>10</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>الصلاة</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -949,6 +1555,30 @@
       <c r="F26" t="n">
         <v>26</v>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>فَٱنتَشِرُواْ</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>62</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>10</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>فانتشروا</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -969,6 +1599,30 @@
       <c r="F27" t="n">
         <v>27</v>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>فِي</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>62</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>10</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>في</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -989,6 +1643,30 @@
       <c r="F28" t="n">
         <v>28</v>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>ٱلۡأَرۡضِ</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>62</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>10</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>الأرض</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1009,6 +1687,30 @@
       <c r="F29" t="n">
         <v>29</v>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>وَٱبۡتَغُواْ</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>62</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>10</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>وابتغوا</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1029,6 +1731,30 @@
       <c r="F30" t="n">
         <v>30</v>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>مِن</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>62</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>10</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>من</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1049,6 +1775,30 @@
       <c r="F31" t="n">
         <v>31</v>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>فَضۡلِ</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>62</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>10</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>فضل</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1069,6 +1819,30 @@
       <c r="F32" t="n">
         <v>32</v>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>ٱللَّهِ</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>62</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>10</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>الله</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1089,6 +1863,30 @@
       <c r="F33" t="n">
         <v>33</v>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>وَٱذۡكُرُواْ</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>62</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>10</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>واذكروا</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1109,6 +1907,30 @@
       <c r="F34" t="n">
         <v>34</v>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>ٱللَّهَ</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>62</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>10</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>الله</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1129,6 +1951,30 @@
       <c r="F35" t="n">
         <v>35</v>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>كَثِيرٗا</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>62</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>10</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>كثيرا</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1149,6 +1995,30 @@
       <c r="F36" t="n">
         <v>36</v>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>لَّعَلَّكُمۡ</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>62</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>10</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>لعلكم</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1169,6 +2039,30 @@
       <c r="F37" t="n">
         <v>37</v>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>تُفۡلِحُونَ</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>62</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>10</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>تفلحون</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1189,6 +2083,30 @@
       <c r="F38" t="n">
         <v>38</v>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>وَإِذَا</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>62</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>11</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>وإذا</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1209,6 +2127,30 @@
       <c r="F39" t="n">
         <v>39</v>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>رَأَوۡاْ</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>62</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>11</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>رأوا</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1229,6 +2171,30 @@
       <c r="F40" t="n">
         <v>40</v>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>تِجَٰرَةً</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>62</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>11</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>تجارة</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1249,6 +2215,30 @@
       <c r="F41" t="n">
         <v>41</v>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>أَوۡ</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>62</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>11</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>أو</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1269,6 +2259,30 @@
       <c r="F42" t="n">
         <v>42</v>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>لَهۡوًا</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>62</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>11</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>لهوا</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1289,6 +2303,30 @@
       <c r="F43" t="n">
         <v>43</v>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>ٱنفَضُّوٓاْ</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>62</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>11</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>انفضوا</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1309,6 +2347,30 @@
       <c r="F44" t="n">
         <v>44</v>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>إِلَيۡهَا</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>62</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>11</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>إليها</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1329,6 +2391,30 @@
       <c r="F45" t="n">
         <v>45</v>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>وَتَرَكُوكَ</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>62</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>11</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>وتركوك</t>
+        </is>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1349,6 +2435,30 @@
       <c r="F46" t="n">
         <v>46</v>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>قَآئِمٗاۚ</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>62</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>11</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>قائما</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1369,6 +2479,30 @@
       <c r="F47" t="n">
         <v>47</v>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>قُلۡ</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>62</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>11</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>قل</t>
+        </is>
+      </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1389,6 +2523,30 @@
       <c r="F48" t="n">
         <v>48</v>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>مَا</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>62</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>11</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ما</t>
+        </is>
+      </c>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1409,6 +2567,30 @@
       <c r="F49" t="n">
         <v>49</v>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>عِندَ</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>62</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>11</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>عند</t>
+        </is>
+      </c>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1429,6 +2611,30 @@
       <c r="F50" t="n">
         <v>50</v>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>ٱللَّهِ</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>62</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>11</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>الله</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1449,6 +2655,30 @@
       <c r="F51" t="n">
         <v>51</v>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>خَيۡرٞ</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>62</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>11</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>خير</t>
+        </is>
+      </c>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1469,6 +2699,30 @@
       <c r="F52" t="n">
         <v>52</v>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>مِّنَ</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>62</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>11</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>من</t>
+        </is>
+      </c>
+      <c r="L52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1489,6 +2743,30 @@
       <c r="F53" t="n">
         <v>53</v>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>ٱللَّهۡوِ</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>62</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>11</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>اللهو</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1509,6 +2787,30 @@
       <c r="F54" t="n">
         <v>54</v>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>وَمِنَ</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>62</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>11</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ومن</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1529,6 +2831,30 @@
       <c r="F55" t="n">
         <v>55</v>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>ٱلتِّجَٰرَةِۚ</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>62</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>11</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>التجارة</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1549,6 +2875,30 @@
       <c r="F56" t="n">
         <v>56</v>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>وَٱللَّهُ</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>62</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>11</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>والله</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1569,6 +2919,30 @@
       <c r="F57" t="n">
         <v>57</v>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>خَيۡرُ</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>62</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>11</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>خير</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1589,6 +2963,30 @@
       <c r="F58" t="n">
         <v>58</v>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>ٱلرَّٰزِقِينَ</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>62</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>الجُمعَة</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>11</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>الرازقين</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1609,6 +3007,30 @@
       <c r="F59" t="n">
         <v>59</v>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>إِذَا</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>63</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>إذا</t>
+        </is>
+      </c>
+      <c r="L59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1629,6 +3051,30 @@
       <c r="F60" t="n">
         <v>60</v>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>جَآءَكَ</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>63</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>1</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>جاءك</t>
+        </is>
+      </c>
+      <c r="L60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1649,6 +3095,30 @@
       <c r="F61" t="n">
         <v>61</v>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>ٱلۡمُنَٰفِقُونَ</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>63</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>1</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>المنافقون</t>
+        </is>
+      </c>
+      <c r="L61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1669,6 +3139,30 @@
       <c r="F62" t="n">
         <v>62</v>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>قَالُواْ</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>63</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>1</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>قالوا</t>
+        </is>
+      </c>
+      <c r="L62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1689,6 +3183,30 @@
       <c r="F63" t="n">
         <v>63</v>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>نَشۡهَدُ</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>63</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>نشهد</t>
+        </is>
+      </c>
+      <c r="L63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1709,6 +3227,30 @@
       <c r="F64" t="n">
         <v>64</v>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>إِنَّكَ</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>63</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>1</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>إنك</t>
+        </is>
+      </c>
+      <c r="L64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1729,6 +3271,30 @@
       <c r="F65" t="n">
         <v>65</v>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>لَرَسُولُ</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>63</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>1</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>لرسول</t>
+        </is>
+      </c>
+      <c r="L65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1749,6 +3315,30 @@
       <c r="F66" t="n">
         <v>66</v>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>ٱللَّهِۗ</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>63</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>1</v>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>الله</t>
+        </is>
+      </c>
+      <c r="L66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1769,6 +3359,30 @@
       <c r="F67" t="n">
         <v>67</v>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>وَٱللَّهُ</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>63</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>1</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>والله</t>
+        </is>
+      </c>
+      <c r="L67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1789,6 +3403,30 @@
       <c r="F68" t="n">
         <v>68</v>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>يَعۡلَمُ</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>63</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>1</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>يعلم</t>
+        </is>
+      </c>
+      <c r="L68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1809,6 +3447,30 @@
       <c r="F69" t="n">
         <v>69</v>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>إِنَّكَ</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>63</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>1</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>إنك</t>
+        </is>
+      </c>
+      <c r="L69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1829,6 +3491,30 @@
       <c r="F70" t="n">
         <v>70</v>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>لَرَسُولُهُۥ</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>63</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>لرسوله</t>
+        </is>
+      </c>
+      <c r="L70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1849,6 +3535,30 @@
       <c r="F71" t="n">
         <v>71</v>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>وَٱللَّهُ</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>63</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>والله</t>
+        </is>
+      </c>
+      <c r="L71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1869,6 +3579,30 @@
       <c r="F72" t="n">
         <v>72</v>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>يَشۡهَدُ</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>63</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>1</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>يشهد</t>
+        </is>
+      </c>
+      <c r="L72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1889,6 +3623,30 @@
       <c r="F73" t="n">
         <v>73</v>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>إِنَّ</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>63</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>1</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>إن</t>
+        </is>
+      </c>
+      <c r="L73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1909,6 +3667,30 @@
       <c r="F74" t="n">
         <v>74</v>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>ٱلۡمُنَٰفِقِينَ</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>63</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>1</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>المنافقين</t>
+        </is>
+      </c>
+      <c r="L74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1929,6 +3711,30 @@
       <c r="F75" t="n">
         <v>75</v>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>لَكَٰذِبُونَ</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>63</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>1</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>لكاذبون</t>
+        </is>
+      </c>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1949,6 +3755,30 @@
       <c r="F76" t="n">
         <v>76</v>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>ٱتَّخَذُوٓاْ</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>63</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>2</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>اتخذوا</t>
+        </is>
+      </c>
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1969,6 +3799,30 @@
       <c r="F77" t="n">
         <v>77</v>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>أَيۡمَٰنَهُمۡ</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>63</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>أيمانهم</t>
+        </is>
+      </c>
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1989,6 +3843,30 @@
       <c r="F78" t="n">
         <v>78</v>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>جُنَّةٗ</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>63</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>2</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>جنة</t>
+        </is>
+      </c>
+      <c r="L78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2009,6 +3887,30 @@
       <c r="F79" t="n">
         <v>79</v>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>فَصَدُّواْ</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>63</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>2</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>فصدوا</t>
+        </is>
+      </c>
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2029,6 +3931,30 @@
       <c r="F80" t="n">
         <v>80</v>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>عَن</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>63</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>2</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>عن</t>
+        </is>
+      </c>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2049,6 +3975,30 @@
       <c r="F81" t="n">
         <v>81</v>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>سَبِيلِ</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
+        <v>63</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>2</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>سبيل</t>
+        </is>
+      </c>
+      <c r="L81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2069,6 +4019,30 @@
       <c r="F82" t="n">
         <v>82</v>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>ٱللَّهِۚ</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>63</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>2</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>الله</t>
+        </is>
+      </c>
+      <c r="L82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2089,6 +4063,30 @@
       <c r="F83" t="n">
         <v>83</v>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>إِنَّهُمۡ</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>63</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>2</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>إنهم</t>
+        </is>
+      </c>
+      <c r="L83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2109,6 +4107,30 @@
       <c r="F84" t="n">
         <v>84</v>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>سَآءَ</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>63</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>2</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ساء</t>
+        </is>
+      </c>
+      <c r="L84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2129,6 +4151,30 @@
       <c r="F85" t="n">
         <v>85</v>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>مَا</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>63</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>2</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ما</t>
+        </is>
+      </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2149,6 +4195,30 @@
       <c r="F86" t="n">
         <v>86</v>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>كَانُواْ</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>63</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>2</v>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>كانوا</t>
+        </is>
+      </c>
+      <c r="L86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2169,6 +4239,30 @@
       <c r="F87" t="n">
         <v>87</v>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>يَعۡمَلُونَ</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>63</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>2</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>يعملون</t>
+        </is>
+      </c>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2189,6 +4283,30 @@
       <c r="F88" t="n">
         <v>89</v>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>ذَٰلِكَ</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>63</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>3</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ذلك</t>
+        </is>
+      </c>
+      <c r="L88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2209,6 +4327,30 @@
       <c r="F89" t="n">
         <v>90</v>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>بِأَنَّهُمۡ</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>63</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>3</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>بأنهم</t>
+        </is>
+      </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2229,6 +4371,30 @@
       <c r="F90" t="n">
         <v>91</v>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>ءَامَنُواْ</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>63</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>3</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>آمنوا</t>
+        </is>
+      </c>
+      <c r="L90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2249,6 +4415,30 @@
       <c r="F91" t="n">
         <v>92</v>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>ثُمَّ</t>
+        </is>
+      </c>
+      <c r="H91" t="n">
+        <v>63</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>3</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ثم</t>
+        </is>
+      </c>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2269,6 +4459,30 @@
       <c r="F92" t="n">
         <v>93</v>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>كَفَرُواْ</t>
+        </is>
+      </c>
+      <c r="H92" t="n">
+        <v>63</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>3</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>كفروا</t>
+        </is>
+      </c>
+      <c r="L92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2289,6 +4503,30 @@
       <c r="F93" t="n">
         <v>94</v>
       </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>فَطُبِعَ</t>
+        </is>
+      </c>
+      <c r="H93" t="n">
+        <v>63</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>3</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>فطبع</t>
+        </is>
+      </c>
+      <c r="L93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2309,6 +4547,30 @@
       <c r="F94" t="n">
         <v>95</v>
       </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>عَلَىٰ</t>
+        </is>
+      </c>
+      <c r="H94" t="n">
+        <v>63</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>3</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>على</t>
+        </is>
+      </c>
+      <c r="L94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2329,6 +4591,30 @@
       <c r="F95" t="n">
         <v>96</v>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>قُلُوبِهِمۡ</t>
+        </is>
+      </c>
+      <c r="H95" t="n">
+        <v>63</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J95" t="n">
+        <v>3</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>قلوبهم</t>
+        </is>
+      </c>
+      <c r="L95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2349,6 +4635,30 @@
       <c r="F96" t="n">
         <v>97</v>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>فَهُمۡ</t>
+        </is>
+      </c>
+      <c r="H96" t="n">
+        <v>63</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J96" t="n">
+        <v>3</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>فهم</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2369,6 +4679,30 @@
       <c r="F97" t="n">
         <v>98</v>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>لَا</t>
+        </is>
+      </c>
+      <c r="H97" t="n">
+        <v>63</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J97" t="n">
+        <v>3</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+      <c r="L97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2389,6 +4723,30 @@
       <c r="F98" t="n">
         <v>99</v>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>يَفۡقَهُونَ</t>
+        </is>
+      </c>
+      <c r="H98" t="n">
+        <v>63</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>3</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>يفقهون</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2409,6 +4767,30 @@
       <c r="F99" t="n">
         <v>124</v>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>وَإِذَا</t>
+        </is>
+      </c>
+      <c r="H99" t="n">
+        <v>63</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>4</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>وإذا</t>
+        </is>
+      </c>
+      <c r="L99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2429,6 +4811,30 @@
       <c r="F100" t="n">
         <v>101</v>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>رَأَيۡتَهُمۡ</t>
+        </is>
+      </c>
+      <c r="H100" t="n">
+        <v>63</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>4</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>رأيتهم</t>
+        </is>
+      </c>
+      <c r="L100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2449,6 +4855,30 @@
       <c r="F101" t="n">
         <v>102</v>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>تُعۡجِبُكَ</t>
+        </is>
+      </c>
+      <c r="H101" t="n">
+        <v>63</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>4</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>تعجبك</t>
+        </is>
+      </c>
+      <c r="L101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2469,6 +4899,30 @@
       <c r="F102" t="n">
         <v>103</v>
       </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>أَجۡسَامُهُمۡۖ</t>
+        </is>
+      </c>
+      <c r="H102" t="n">
+        <v>63</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>4</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>أجسامهم</t>
+        </is>
+      </c>
+      <c r="L102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2489,6 +4943,30 @@
       <c r="F103" t="n">
         <v>104</v>
       </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>وَإِن</t>
+        </is>
+      </c>
+      <c r="H103" t="n">
+        <v>63</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>4</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>وإن</t>
+        </is>
+      </c>
+      <c r="L103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -2509,6 +4987,30 @@
       <c r="F104" t="n">
         <v>105</v>
       </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>يَقُولُواْ</t>
+        </is>
+      </c>
+      <c r="H104" t="n">
+        <v>63</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>4</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>يقولوا</t>
+        </is>
+      </c>
+      <c r="L104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2529,6 +5031,30 @@
       <c r="F105" t="n">
         <v>106</v>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>تَسۡمَعۡ</t>
+        </is>
+      </c>
+      <c r="H105" t="n">
+        <v>63</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>4</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>تسمع</t>
+        </is>
+      </c>
+      <c r="L105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2549,6 +5075,30 @@
       <c r="F106" t="n">
         <v>107</v>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>لِقَوۡلِهِمۡۖ</t>
+        </is>
+      </c>
+      <c r="H106" t="n">
+        <v>63</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>4</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>لقولهم</t>
+        </is>
+      </c>
+      <c r="L106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2569,6 +5119,30 @@
       <c r="F107" t="n">
         <v>108</v>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>كَأَنَّهُمۡ</t>
+        </is>
+      </c>
+      <c r="H107" t="n">
+        <v>63</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>4</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>كأنهم</t>
+        </is>
+      </c>
+      <c r="L107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2589,6 +5163,30 @@
       <c r="F108" t="n">
         <v>109</v>
       </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>خُشُبٞ</t>
+        </is>
+      </c>
+      <c r="H108" t="n">
+        <v>63</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>4</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>خشب</t>
+        </is>
+      </c>
+      <c r="L108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2609,6 +5207,30 @@
       <c r="F109" t="n">
         <v>110</v>
       </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>مُّسَنَّدَةٞۖ</t>
+        </is>
+      </c>
+      <c r="H109" t="n">
+        <v>63</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>4</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>مسندة</t>
+        </is>
+      </c>
+      <c r="L109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -2629,6 +5251,30 @@
       <c r="F110" t="n">
         <v>111</v>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>يَحۡسَبُونَ</t>
+        </is>
+      </c>
+      <c r="H110" t="n">
+        <v>63</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>4</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>يحسبون</t>
+        </is>
+      </c>
+      <c r="L110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -2649,6 +5295,30 @@
       <c r="F111" t="n">
         <v>112</v>
       </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>كُلَّ</t>
+        </is>
+      </c>
+      <c r="H111" t="n">
+        <v>63</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>4</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>كل</t>
+        </is>
+      </c>
+      <c r="L111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2669,6 +5339,30 @@
       <c r="F112" t="n">
         <v>113</v>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>صَيۡحَةٍ</t>
+        </is>
+      </c>
+      <c r="H112" t="n">
+        <v>63</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>4</v>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>صيحة</t>
+        </is>
+      </c>
+      <c r="L112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -2689,6 +5383,30 @@
       <c r="F113" t="n">
         <v>114</v>
       </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>عَلَيۡهِمۡۚ</t>
+        </is>
+      </c>
+      <c r="H113" t="n">
+        <v>63</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>4</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>عليهم</t>
+        </is>
+      </c>
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -2709,6 +5427,30 @@
       <c r="F114" t="n">
         <v>115</v>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>هُمُ</t>
+        </is>
+      </c>
+      <c r="H114" t="n">
+        <v>63</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>4</v>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>هم</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -2729,6 +5471,30 @@
       <c r="F115" t="n">
         <v>116</v>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>ٱلۡعَدُوُّ</t>
+        </is>
+      </c>
+      <c r="H115" t="n">
+        <v>63</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>4</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>العدو</t>
+        </is>
+      </c>
+      <c r="L115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -2749,6 +5515,30 @@
       <c r="F116" t="n">
         <v>117</v>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>فَٱحۡذَرۡهُمۡۚ</t>
+        </is>
+      </c>
+      <c r="H116" t="n">
+        <v>63</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>4</v>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>فاحذرهم</t>
+        </is>
+      </c>
+      <c r="L116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -2769,6 +5559,30 @@
       <c r="F117" t="n">
         <v>118</v>
       </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>قَٰتَلَهُمُ</t>
+        </is>
+      </c>
+      <c r="H117" t="n">
+        <v>63</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>4</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>قاتلهم</t>
+        </is>
+      </c>
+      <c r="L117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -2789,6 +5603,30 @@
       <c r="F118" t="n">
         <v>119</v>
       </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>ٱللَّهُۖ</t>
+        </is>
+      </c>
+      <c r="H118" t="n">
+        <v>63</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J118" t="n">
+        <v>4</v>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>الله</t>
+        </is>
+      </c>
+      <c r="L118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -2809,6 +5647,30 @@
       <c r="F119" t="n">
         <v>120</v>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>أَنَّىٰ</t>
+        </is>
+      </c>
+      <c r="H119" t="n">
+        <v>63</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J119" t="n">
+        <v>4</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>أنى</t>
+        </is>
+      </c>
+      <c r="L119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -2828,6 +5690,30 @@
       </c>
       <c r="F120" t="n">
         <v>121</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>يُؤۡفَكُونَ</t>
+        </is>
+      </c>
+      <c r="H120" t="n">
+        <v>63</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>المُنَافِقُونَ</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
+        <v>4</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>يؤفكون</t>
+        </is>
+      </c>
+      <c r="L120" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>